<commit_message>
maxinum in maximum in xls file
</commit_message>
<xml_diff>
--- a/static/files/logements.xlsx
+++ b/static/files/logements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolasoudard/workspace/beta.gouv.fr/apilos/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3FCFED-12B3-4140-8933-88B3408D72CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010CD73E-B016-E748-92F2-005EE1D5224B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34480" yWindow="4440" windowWidth="27020" windowHeight="16440" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
+    <workbookView xWindow="1000" yWindow="500" windowWidth="27800" windowHeight="17500" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Logements" sheetId="1" r:id="rId1"/>
@@ -117,23 +117,23 @@
 (article R.111-2)</t>
   </si>
   <si>
-    <t>Loyer maxinum en € par m² de surface utile</t>
-  </si>
-  <si>
-    <t>Loyer maxinum du logement en €
+    <t>2. Modifier à votre guise le fichier</t>
+  </si>
+  <si>
+    <t>5. Vérifier le contenu téléversé dans l'application et enregistrer en cliquant sur le bouton 'Enregistrer et Suivant'</t>
+  </si>
+  <si>
+    <t>Attention : ne pas mettre la ligne Total dans ce tableau</t>
+  </si>
+  <si>
+    <t>elle sera calculée automatiquement lors de l'import des logements</t>
+  </si>
+  <si>
+    <t>Loyer maximum en € par m² de surface utile</t>
+  </si>
+  <si>
+    <t>Loyer maximum du logement en €
 (col 4 * col 5 * col 6)</t>
-  </si>
-  <si>
-    <t>2. Modifier à votre guise le fichier</t>
-  </si>
-  <si>
-    <t>5. Vérifier le contenu téléversé dans l'application et enregistrer en cliquant sur le bouton 'Enregistrer et Suivant'</t>
-  </si>
-  <si>
-    <t>Attention : ne pas mettre la ligne Total dans ce tableau</t>
-  </si>
-  <si>
-    <t>elle sera calculée automatiquement lors de l'import des logements</t>
   </si>
 </sst>
 </file>
@@ -362,13 +362,13 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,27 +788,27 @@
         <v>21</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H1" s="16" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="19" x14ac:dyDescent="0.25">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="33"/>
+      <c r="B2" s="34"/>
       <c r="C2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="33"/>
+      <c r="E2" s="34"/>
       <c r="F2" s="13" t="s">
         <v>16</v>
       </c>
@@ -821,8 +821,8 @@
       <c r="I2" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="34" t="s">
-        <v>29</v>
+      <c r="J2" s="32" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -836,7 +836,7 @@
       <c r="H3" s="29"/>
       <c r="I3" s="24"/>
       <c r="J3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -1426,7 +1426,7 @@
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.2">
@@ -1441,7 +1441,7 @@
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
WIP adapter les avenants aux convention mixte
</commit_message>
<xml_diff>
--- a/static/files/logements.xlsx
+++ b/static/files/logements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayoub.bouchachia\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\production\siap\apilos\static\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B9CB336-2071-427E-BEF6-2274AED39178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F55035CC-1F0E-448F-937F-8571E355743A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16110" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Logements" sheetId="1" r:id="rId1"/>
@@ -71,95 +71,95 @@
     <t>Coefficient propre au logement</t>
   </si>
   <si>
+    <t>(Utilisez votre propre nomenclature, elle doit correspondre à celle indiquée dans l’EDD simplifié, ex : 604, Bâtiment B, étage 4, escalier 3, logement N°604)</t>
+  </si>
+  <si>
+    <t>Par défaut, indiquez un coefficient de 1 si vous n’appliquez pas de pondération particulière)</t>
+  </si>
+  <si>
+    <t>Col 1</t>
+  </si>
+  <si>
+    <t>Col 2</t>
+  </si>
+  <si>
+    <t>Col 3</t>
+  </si>
+  <si>
+    <t>Col 4</t>
+  </si>
+  <si>
+    <t>Col 5</t>
+  </si>
+  <si>
+    <t>Col 6</t>
+  </si>
+  <si>
+    <t>Col 7</t>
+  </si>
+  <si>
+    <t>Col 8</t>
+  </si>
+  <si>
+    <t>Attention : ne pas mettre la ligne Total dans ce tableau</t>
+  </si>
+  <si>
+    <t>elle sera calculée automatiquement lors de l'import des logements</t>
+  </si>
+  <si>
+    <t>Ici quelques explications</t>
+  </si>
+  <si>
+    <t>1. Telechager le modèle (ce fichier)</t>
+  </si>
+  <si>
+    <t>2. Modifier à votre guise le fichier</t>
+  </si>
+  <si>
+    <t>3. Enregistrer vos modifications</t>
+  </si>
+  <si>
+    <t>4. Téléverser le fichier modifié dans l'application</t>
+  </si>
+  <si>
+    <t>5. Vérifier le contenu téléversé dans l'application et enregistrer en cliquant sur le bouton 'Enregistrer et Suivant'</t>
+  </si>
+  <si>
+    <t>Attention, en aucun cas vous ne devez modifier l'entête du tableau des prêts, cela casserait l'import des données</t>
+  </si>
+  <si>
+    <t>Type de logement</t>
+  </si>
+  <si>
+    <t>lignes data</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>T1bis</t>
+  </si>
+  <si>
+    <t>T1'</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>T3</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>T6 et plus</t>
+  </si>
+  <si>
     <t>Loyer maximum du logement en €
-(col 4 * col 5 * col 6)</t>
-  </si>
-  <si>
-    <t>(Utilisez votre propre nomenclature, elle doit correspondre à celle indiquée dans l’EDD simplifié, ex : 604, Bâtiment B, étage 4, escalier 3, logement N°604)</t>
-  </si>
-  <si>
-    <t>Par défaut, indiquez un coefficient de 1 si vous n’appliquez pas de pondération particulière)</t>
-  </si>
-  <si>
-    <t>Col 1</t>
-  </si>
-  <si>
-    <t>Col 2</t>
-  </si>
-  <si>
-    <t>Col 3</t>
-  </si>
-  <si>
-    <t>Col 4</t>
-  </si>
-  <si>
-    <t>Col 5</t>
-  </si>
-  <si>
-    <t>Col 6</t>
-  </si>
-  <si>
-    <t>Col 7</t>
-  </si>
-  <si>
-    <t>Col 8</t>
-  </si>
-  <si>
-    <t>Attention : ne pas mettre la ligne Total dans ce tableau</t>
-  </si>
-  <si>
-    <t>elle sera calculée automatiquement lors de l'import des logements</t>
-  </si>
-  <si>
-    <t>Ici quelques explications</t>
-  </si>
-  <si>
-    <t>1. Telechager le modèle (ce fichier)</t>
-  </si>
-  <si>
-    <t>2. Modifier à votre guise le fichier</t>
-  </si>
-  <si>
-    <t>3. Enregistrer vos modifications</t>
-  </si>
-  <si>
-    <t>4. Téléverser le fichier modifié dans l'application</t>
-  </si>
-  <si>
-    <t>5. Vérifier le contenu téléversé dans l'application et enregistrer en cliquant sur le bouton 'Enregistrer et Suivant'</t>
-  </si>
-  <si>
-    <t>Attention, en aucun cas vous ne devez modifier l'entête du tableau des prêts, cela casserait l'import des données</t>
-  </si>
-  <si>
-    <t>Type de logement</t>
-  </si>
-  <si>
-    <t>lignes data</t>
-  </si>
-  <si>
-    <t>T1</t>
-  </si>
-  <si>
-    <t>T1bis</t>
-  </si>
-  <si>
-    <t>T1'</t>
-  </si>
-  <si>
-    <t>T2</t>
-  </si>
-  <si>
-    <t>T3</t>
-  </si>
-  <si>
-    <t>T4</t>
-  </si>
-  <si>
-    <t>T5</t>
-  </si>
-  <si>
-    <t>T6 et plus</t>
+(col 5 * col 6 * col 7)</t>
   </si>
 </sst>
 </file>
@@ -875,12 +875,12 @@
         <v>8</v>
       </c>
       <c r="J1" s="37" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -890,39 +890,39 @@
       <c r="G2" s="36"/>
       <c r="H2" s="36"/>
       <c r="I2" s="28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J2" s="38"/>
     </row>
     <row r="3" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="34"/>
       <c r="C3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="34" t="s">
         <v>14</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>15</v>
       </c>
       <c r="F3" s="34"/>
       <c r="G3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="I3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="J3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="K3" s="20" t="s">
         <v>19</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -937,7 +937,7 @@
       <c r="I4" s="21"/>
       <c r="J4" s="24"/>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -1712,37 +1712,37 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1761,15 +1761,15 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="29" t="s">
         <v>29</v>
-      </c>
-      <c r="E1" s="29" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="30">
         <v>4</v>
@@ -1777,39 +1777,39 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E3" s="31"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>